<commit_message>
office: update AMAVIO final artifacts and coach package
</commit_message>
<xml_diff>
--- a/04_Final_Abgabe_v2_1/02_Finanzmodell/AMAVIO_Finanzmodell_36_Monate_v1_8_FINAL.xlsx
+++ b/04_Final_Abgabe_v2_1/02_Finanzmodell/AMAVIO_Finanzmodell_36_Monate_v1_8_FINAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zakia\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f1f35f86780e4cd/Desktop/04_Final_Abgabe_v2_1/02_Finanzmodell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73665839-8173-4CFE-80B2-2EA4ABA11D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{73665839-8173-4CFE-80B2-2EA4ABA11D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2240AA1F-F1B3-4E00-B78D-1E5C3214B9D6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,6 @@
     <sheet name="Dashboard" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029" forceFullCalc="1"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -47,17 +46,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="416">
-  <si>
-    <t>AMAVIO | Finanzmodell 36 Monate v1.7 FINAL</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="415">
   <si>
     <t>Finale Baseline: dynamische Zahlungspläne, Plan-/Live-Liquidität, Steuerreserven, Szenarien und Modellchecks</t>
   </si>
   <si>
-    <t>Kernfassung 1.7 · AMAVIO Living · Preis-, Cash- und Quellen-Synchronisierung · 28. Juli 2026</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -109,9 +102,6 @@
     <t>28. Juli 2026</t>
   </si>
   <si>
-    <t>AMAVIO Source of Truth v2.1</t>
-  </si>
-  <si>
     <t>Item</t>
   </si>
   <si>
@@ -169,9 +159,6 @@
     <t>EBITDA Jahr 3</t>
   </si>
   <si>
-    <t>AMAVIO Förder- und Finanzierungsbausteine v2.1</t>
-  </si>
-  <si>
     <t>Baustein</t>
   </si>
   <si>
@@ -311,9 +298,6 @@
   </si>
   <si>
     <t>BMF LStH/SvEV</t>
-  </si>
-  <si>
-    <t>AMAVIO Cash Timing Stress v2.1</t>
   </si>
   <si>
     <t>Stress</t>
@@ -1018,9 +1002,6 @@
     <t>AMAVIO | Modellchecks und Freigabestatus</t>
   </si>
   <si>
-    <t>PASS setzt fehlerfreie Formeln sowie dokumentierte Startfinanzierung voraus; andernfalls bleibt das Modell CONDITIONAL.</t>
-  </si>
-  <si>
     <t>Check</t>
   </si>
   <si>
@@ -1096,9 +1077,6 @@
     <t>Live cash roll-forward</t>
   </si>
   <si>
-    <t>Formula error scan</t>
-  </si>
-  <si>
     <t>Final external scan required</t>
   </si>
   <si>
@@ -1198,24 +1176,15 @@
     <t>Internal baseline</t>
   </si>
   <si>
-    <t>Businessplan Kernfassung v1.7, chapter 9</t>
-  </si>
-  <si>
     <t>EUR net</t>
   </si>
   <si>
-    <t>Businessplan v1.7; P0 Commercial Architecture</t>
-  </si>
-  <si>
     <t>29,500 EUR is the binding Launch baseline; no reduced Launch price is used in the model</t>
   </si>
   <si>
     <t>Internal calibration</t>
   </si>
   <si>
-    <t>Businessplan v1.7, chapters 1 and 8</t>
-  </si>
-  <si>
     <t>Not a market statistic</t>
   </si>
   <si>
@@ -1225,9 +1194,6 @@
     <t>Internal policy</t>
   </si>
   <si>
-    <t>Businessplan v1.7, payment model</t>
-  </si>
-  <si>
     <t>Order / system approval / go-live</t>
   </si>
   <si>
@@ -1237,9 +1203,6 @@
     <t>Internal financing plan</t>
   </si>
   <si>
-    <t>Businessplan v1.7 and evidence package</t>
-  </si>
-  <si>
     <t>500 EUR share capital + 24,500 EUR documented contribution/loan</t>
   </si>
   <si>
@@ -1249,15 +1212,9 @@
     <t>Planning assumption</t>
   </si>
   <si>
-    <t>Businessplan v1.7, chapter 9</t>
-  </si>
-  <si>
     <t>Not a tax calculation; tax adviser to confirm</t>
   </si>
   <si>
-    <t>AMAVIO | Managementübersicht – Baseline v1.7</t>
-  </si>
-  <si>
     <t>Plan- und Live-Sicht bleiben bewusst getrennt. Der Live-Status reagiert auf den dokumentierten Finanzierungszufluss in Assumptions.</t>
   </si>
   <si>
@@ -1304,6 +1261,45 @@
   </si>
   <si>
     <t>Month</t>
+  </si>
+  <si>
+    <t>AMAVIO | Finanzmodell 36 Monate v1.8 FINAL</t>
+  </si>
+  <si>
+    <t>Kernfassung 1.8 · AMAVIO Living · Preis-, Cash- und Quellen-Synchronisierung · 30. Juli 2026</t>
+  </si>
+  <si>
+    <t>AMAVIO | Managementübersicht · Baseline v1.8</t>
+  </si>
+  <si>
+    <t>PASS setzt fehlerfreie Kernformeln, vollständige Startfinanzierung, Mindestliquidität und geschlossene P1-Gates voraus; andernfalls bleibt das Modell CONDITIONAL.</t>
+  </si>
+  <si>
+    <t>Key formula error scan</t>
+  </si>
+  <si>
+    <t>AMAVIO Source of Truth v2.2</t>
+  </si>
+  <si>
+    <t>AMAVIO Förder- und Finanzierungsbausteine v2.2</t>
+  </si>
+  <si>
+    <t>AMAVIO Cash Timing Stress v2.2</t>
+  </si>
+  <si>
+    <t>Businessplan Master v2.2, Kapitel 9</t>
+  </si>
+  <si>
+    <t>Businessplan Master v2.2; P0 Commercial Architecture</t>
+  </si>
+  <si>
+    <t>Businessplan Master v2.2, Kapitel 1 und 8</t>
+  </si>
+  <si>
+    <t>Businessplan Master v2.2, Zahlungsmodell</t>
+  </si>
+  <si>
+    <t>Businessplan Master v2.2 und Nachweispaket v2.2</t>
   </si>
 </sst>
 </file>
@@ -2101,7 +2097,7 @@
             <c:numRef>
               <c:f>Dashboard!$B$14:$B$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>93500</c:v>
@@ -2155,7 +2151,7 @@
             <c:numRef>
               <c:f>Dashboard!$C$14:$C$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>34950</c:v>
@@ -2209,7 +2205,7 @@
             <c:numRef>
               <c:f>Dashboard!$D$14:$D$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>23065</c:v>
@@ -2480,7 +2476,7 @@
             <c:numRef>
               <c:f>Dashboard!$B$20:$B$55</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
                   <c:v>18576.25</c:v>
@@ -2734,7 +2730,7 @@
             <c:numRef>
               <c:f>Dashboard!$C$20:$C$55</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
                   <c:v>-6423.75</c:v>
@@ -2988,7 +2984,7 @@
             <c:numRef>
               <c:f>Dashboard!$D$20:$D$55</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>\€#,##0;[Red]\(\€#,##0\);\-</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
                   <c:v>10000</c:v>
@@ -3283,6 +3279,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3489,7 +3489,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="20">
       <c r="A1" s="87" t="s">
-        <v>0</v>
+        <v>402</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -3501,7 +3501,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="85" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -3514,7 +3514,7 @@
     <row r="3" spans="1:8">
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>403</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -3525,7 +3525,7 @@
     </row>
     <row r="4" spans="1:8" ht="28" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="4" t="str">
         <f>Checks!E18</f>
@@ -3540,10 +3540,10 @@
     </row>
     <row r="5" spans="1:8" ht="28" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -3554,10 +3554,10 @@
     </row>
     <row r="6" spans="1:8" ht="28" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -3568,10 +3568,10 @@
     </row>
     <row r="7" spans="1:8" ht="28" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -3582,10 +3582,10 @@
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -3596,10 +3596,10 @@
     </row>
     <row r="9" spans="1:8" ht="28" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -3610,10 +3610,10 @@
     </row>
     <row r="10" spans="1:8" ht="28" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -3624,10 +3624,10 @@
     </row>
     <row r="11" spans="1:8" ht="28" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -3638,10 +3638,10 @@
     </row>
     <row r="12" spans="1:8" ht="28" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -3673,7 +3673,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28" customHeight="1">
       <c r="A1" s="88" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -3686,7 +3686,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="93" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -3699,36 +3699,36 @@
     </row>
     <row r="3" spans="1:9" ht="42">
       <c r="A3" s="22" t="s">
+        <v>296</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>297</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>299</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>290</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="I3" s="22" t="s">
         <v>301</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>195</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>302</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>303</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>304</v>
-      </c>
-      <c r="F3" s="22" t="s">
-        <v>305</v>
-      </c>
-      <c r="G3" s="22" t="s">
-        <v>295</v>
-      </c>
-      <c r="H3" s="22" t="s">
-        <v>296</v>
-      </c>
-      <c r="I3" s="22" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="45" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B4" s="46">
         <v>1</v>
@@ -3758,12 +3758,12 @@
         <v>0</v>
       </c>
       <c r="I4" s="49" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="50" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B5" s="51">
         <v>2</v>
@@ -3793,12 +3793,12 @@
         <v>0</v>
       </c>
       <c r="I5" s="54" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="50" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B6" s="51">
         <v>3</v>
@@ -3828,12 +3828,12 @@
         <v>0</v>
       </c>
       <c r="I6" s="54" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="55" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B7" s="56">
         <v>1</v>
@@ -3863,12 +3863,12 @@
         <v>9885</v>
       </c>
       <c r="I7" s="58" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="55" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B8" s="56">
         <v>2</v>
@@ -3898,12 +3898,12 @@
         <v>35196</v>
       </c>
       <c r="I8" s="58" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="55" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B9" s="56">
         <v>3</v>
@@ -3933,12 +3933,12 @@
         <v>49290</v>
       </c>
       <c r="I9" s="58" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="59" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B10" s="60">
         <v>1</v>
@@ -3968,12 +3968,12 @@
         <v>16196.25</v>
       </c>
       <c r="I10" s="63" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="59" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B11" s="60">
         <v>2</v>
@@ -4003,12 +4003,12 @@
         <v>52950</v>
       </c>
       <c r="I11" s="63" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="59" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B12" s="60">
         <v>3</v>
@@ -4038,7 +4038,7 @@
         <v>77467.5</v>
       </c>
       <c r="I12" s="63" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -4086,7 +4086,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="88" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -4096,7 +4096,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="93" t="s">
-        <v>320</v>
+        <v>405</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -4106,27 +4106,27 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="22" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="64" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="B4" s="65">
         <f>'Annual_P&amp;L'!B4</f>
@@ -4144,12 +4144,12 @@
         <v>OK</v>
       </c>
       <c r="F4" s="71" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="67" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="B5" s="36">
         <f>'Annual_P&amp;L'!C4</f>
@@ -4167,12 +4167,12 @@
         <v>OK</v>
       </c>
       <c r="F5" s="72" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="67" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B6" s="36">
         <f>'Annual_P&amp;L'!D4</f>
@@ -4190,12 +4190,12 @@
         <v>OK</v>
       </c>
       <c r="F6" s="72" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="67" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="B7" s="36">
         <f>SUM(Contract_Cash!E28:AN28)</f>
@@ -4214,12 +4214,12 @@
         <v>OK</v>
       </c>
       <c r="F7" s="72" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="67" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="B8" s="36">
         <f>SUM(Contract_Cash!E7:AN7)+SUM(Contract_Cash!E15:AN15)+SUM(Contract_Cash!E24:AN25)</f>
@@ -4238,12 +4238,12 @@
         <v>OK</v>
       </c>
       <c r="F8" s="72" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="67" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="B9" s="36">
         <f>Monthly_Cash!B14</f>
@@ -4262,12 +4262,12 @@
         <v>OK</v>
       </c>
       <c r="F9" s="72" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="67" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="B10" s="36">
         <f>Monthly_Cash!B15</f>
@@ -4286,12 +4286,12 @@
         <v>OK</v>
       </c>
       <c r="F10" s="72" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="67" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B11" s="36">
         <f>Assumptions!B17</f>
@@ -4309,12 +4309,12 @@
         <v>OK</v>
       </c>
       <c r="F11" s="72" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="67" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="B12" s="68">
         <f>Scenarios!C4</f>
@@ -4333,12 +4333,12 @@
         <v>OK</v>
       </c>
       <c r="F12" s="72" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="67" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="B13" s="68">
         <f>Scenarios!C10</f>
@@ -4357,12 +4357,12 @@
         <v>OK</v>
       </c>
       <c r="F13" s="72" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="67" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="B14" s="36">
         <f>'Annual_P&amp;L'!B12</f>
@@ -4381,12 +4381,12 @@
         <v>OK</v>
       </c>
       <c r="F14" s="72" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="67" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="B15" s="36">
         <f>Monthly_Cash!AK17</f>
@@ -4405,12 +4405,12 @@
         <v>OK</v>
       </c>
       <c r="F15" s="72" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="67" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="B16" s="36">
         <f>Monthly_Cash!AK19</f>
@@ -4429,14 +4429,15 @@
         <v>OK</v>
       </c>
       <c r="F16" s="72" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="67" t="s">
-        <v>346</v>
+        <v>406</v>
       </c>
       <c r="B17" s="17">
+        <f>SUMPRODUCT(--ISERROR('Annual_P&amp;L'!B4:D13))+SUMPRODUCT(--ISERROR(Monthly_Cash!B7:AK29))+SUMPRODUCT(--ISERROR(Contract_Cash!E7:AN28))+SUMPRODUCT(--ISERROR(Scenarios!B4:H10))</f>
         <v>0</v>
       </c>
       <c r="C17" s="17">
@@ -4451,19 +4452,19 @@
         <v>OK</v>
       </c>
       <c r="F17" s="72" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="28">
       <c r="A18" s="69" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B18" s="70" t="str">
-        <f>IF(COUNTIF(E4:E17,"FAIL")&gt;0,"FAIL",IF(Assumptions!B5&gt;0,"PASS","CONDITIONAL"))</f>
+        <f>IF(COUNTIF(E4:E17,"FAIL")&gt;0,"FAIL",IF(AND(Assumptions!B5&gt;=Assumptions!B4,COUNTIF(Monthly_Cash!B28:AK29,"BELOW MIN")=0,COUNTIF(P1_Gates!D3:D7,"Erledigt")=5,Assumptions!B18="CONFIRMED"),"PASS","CONDITIONAL"))</f>
         <v>CONDITIONAL</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="D18" s="70">
         <f>IF(B18=C18,0,1)</f>
@@ -4474,7 +4475,7 @@
         <v>CONDITIONAL</v>
       </c>
       <c r="F18" s="73" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -4510,7 +4511,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -4520,7 +4521,7 @@
     </row>
     <row r="2" spans="1:6" ht="14.5">
       <c r="A2" s="89" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -4530,33 +4531,33 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="22" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="23" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B4" s="24">
         <v>3</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D4" s="24">
         <v>3</v>
@@ -4565,18 +4566,18 @@
         <v>1</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="26" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B5" s="27">
         <v>6</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D5" s="27">
         <v>3</v>
@@ -4585,18 +4586,18 @@
         <v>1</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="26" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B6" s="27">
         <v>7</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D6" s="27">
         <v>4</v>
@@ -4605,18 +4606,18 @@
         <v>1</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="26" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B7" s="27">
         <v>10</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="D7" s="27">
         <v>3</v>
@@ -4625,18 +4626,18 @@
         <v>1</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="26" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B8" s="27">
         <v>10</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="D8" s="27">
         <v>3</v>
@@ -4645,18 +4646,18 @@
         <v>1</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="26" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B9" s="27">
         <v>10</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="D9" s="27">
         <v>3</v>
@@ -4665,18 +4666,18 @@
         <v>1</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="26" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B10" s="27">
         <v>13</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D10" s="27">
         <v>3</v>
@@ -4685,18 +4686,18 @@
         <v>1</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="26" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B11" s="27">
         <v>16</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D11" s="27">
         <v>3</v>
@@ -4705,18 +4706,18 @@
         <v>1</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="26" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B12" s="27">
         <v>19</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D12" s="27">
         <v>3</v>
@@ -4725,18 +4726,18 @@
         <v>1</v>
       </c>
       <c r="F12" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="26" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B13" s="27">
         <v>14</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D13" s="27">
         <v>4</v>
@@ -4745,18 +4746,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="21" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="26" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B14" s="27">
         <v>18</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D14" s="27">
         <v>4</v>
@@ -4765,18 +4766,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="26" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B15" s="27">
         <v>18</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="D15" s="27">
         <v>3</v>
@@ -4785,18 +4786,18 @@
         <v>1</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="26" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B16" s="27">
         <v>13</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="D16" s="27">
         <v>12</v>
@@ -4805,18 +4806,18 @@
         <v>1</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="26" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B17" s="27">
         <v>17</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="D17" s="27">
         <v>3</v>
@@ -4825,18 +4826,18 @@
         <v>3</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="26" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B18" s="27">
         <v>25</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D18" s="27">
         <v>3</v>
@@ -4845,18 +4846,18 @@
         <v>1</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="26" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B19" s="27">
         <v>27</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D19" s="27">
         <v>3</v>
@@ -4865,18 +4866,18 @@
         <v>1</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="26" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B20" s="27">
         <v>29</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D20" s="27">
         <v>3</v>
@@ -4885,18 +4886,18 @@
         <v>1</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="26" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B21" s="27">
         <v>31</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D21" s="27">
         <v>3</v>
@@ -4905,18 +4906,18 @@
         <v>1</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="26" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B22" s="27">
         <v>25</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D22" s="27">
         <v>4</v>
@@ -4925,18 +4926,18 @@
         <v>1</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="26" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="B23" s="27">
         <v>30</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D23" s="27">
         <v>4</v>
@@ -4945,18 +4946,18 @@
         <v>1</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="26" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B24" s="27">
         <v>27</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="D24" s="27">
         <v>3</v>
@@ -4965,18 +4966,18 @@
         <v>1</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="26" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B25" s="27">
         <v>32</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="D25" s="27">
         <v>3</v>
@@ -4985,18 +4986,18 @@
         <v>1</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="26" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B26" s="27">
         <v>25</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="D26" s="27">
         <v>12</v>
@@ -5005,18 +5006,18 @@
         <v>1</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="26" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B27" s="27">
         <v>25</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="D27" s="27">
         <v>12</v>
@@ -5025,7 +5026,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -5060,7 +5061,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -5078,142 +5079,142 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="22" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="23" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="E4" s="74" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="28">
       <c r="A5" s="26" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B5" s="36">
         <v>29500</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>382</v>
+        <v>411</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="26" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B6" s="36">
         <v>900</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="E6" s="75" t="s">
-        <v>385</v>
+        <v>412</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="26" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="E7" s="75" t="s">
-        <v>389</v>
+        <v>413</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="28">
       <c r="A8" s="26" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="B8" s="36">
         <v>25000</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="E8" s="75" t="s">
-        <v>393</v>
+        <v>414</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="26" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B9" s="68">
         <v>0.3</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="E9" s="75" t="s">
-        <v>397</v>
+        <v>410</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -5236,7 +5237,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="28" customHeight="1">
       <c r="A1" s="94" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -5254,7 +5255,7 @@
     </row>
     <row r="2" spans="1:14" ht="14.5">
       <c r="A2" s="89" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -5288,13 +5289,13 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="22" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
@@ -5310,14 +5311,14 @@
     </row>
     <row r="5" spans="1:14" ht="15.5">
       <c r="A5" s="9" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B5" s="76" t="str">
         <f>Checks!E18</f>
         <v>CONDITIONAL</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="D5" s="34"/>
       <c r="E5" s="34"/>
@@ -5333,14 +5334,14 @@
     </row>
     <row r="6" spans="1:14" ht="15.5">
       <c r="A6" s="15" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="B6" s="77">
         <f>'Annual_P&amp;L'!B4</f>
         <v>93500</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="34"/>
@@ -5356,14 +5357,14 @@
     </row>
     <row r="7" spans="1:14" ht="15.5">
       <c r="A7" s="15" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="B7" s="77">
         <f>'Annual_P&amp;L'!B11</f>
         <v>32950</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="D7" s="34"/>
       <c r="E7" s="34"/>
@@ -5379,14 +5380,14 @@
     </row>
     <row r="8" spans="1:14" ht="15.5">
       <c r="A8" s="15" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="B8" s="77">
         <f>'Annual_P&amp;L'!B13</f>
         <v>23065</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="D8" s="34"/>
       <c r="E8" s="34"/>
@@ -5402,14 +5403,14 @@
     </row>
     <row r="9" spans="1:14" ht="15.5">
       <c r="A9" s="15" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
       <c r="B9" s="77">
         <f>MIN(Monthly_Cash!B26:AK26)</f>
         <v>-792.5</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="D9" s="34"/>
       <c r="E9" s="34"/>
@@ -5425,14 +5426,14 @@
     </row>
     <row r="10" spans="1:14" ht="15.5">
       <c r="A10" s="15" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="B10" s="77">
         <f>MIN(Monthly_Cash!B27:AK27)</f>
         <v>-25792.5</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
@@ -5480,16 +5481,16 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="22" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="E13" s="34"/>
       <c r="F13" s="34"/>
@@ -5617,16 +5618,16 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="22" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="E19" s="34"/>
       <c r="F19" s="34"/>
@@ -5641,7 +5642,7 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="23" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B20" s="78">
         <f>Monthly_Cash!B23</f>
@@ -5668,7 +5669,7 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="26" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B21" s="36">
         <f>Monthly_Cash!C23</f>
@@ -5695,7 +5696,7 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="26" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B22" s="36">
         <f>Monthly_Cash!D23</f>
@@ -5722,7 +5723,7 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="26" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B23" s="36">
         <f>Monthly_Cash!E23</f>
@@ -5749,7 +5750,7 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="26" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B24" s="36">
         <f>Monthly_Cash!F23</f>
@@ -5776,7 +5777,7 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="26" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B25" s="36">
         <f>Monthly_Cash!G23</f>
@@ -5803,7 +5804,7 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="26" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B26" s="36">
         <f>Monthly_Cash!H23</f>
@@ -5830,7 +5831,7 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="26" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B27" s="36">
         <f>Monthly_Cash!I23</f>
@@ -5857,7 +5858,7 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="26" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B28" s="36">
         <f>Monthly_Cash!J23</f>
@@ -5884,7 +5885,7 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="26" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B29" s="36">
         <f>Monthly_Cash!K23</f>
@@ -5911,7 +5912,7 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="26" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B30" s="36">
         <f>Monthly_Cash!L23</f>
@@ -5938,7 +5939,7 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="26" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B31" s="36">
         <f>Monthly_Cash!M23</f>
@@ -5965,7 +5966,7 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="26" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B32" s="36">
         <f>Monthly_Cash!N23</f>
@@ -5992,7 +5993,7 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="26" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="B33" s="36">
         <f>Monthly_Cash!O23</f>
@@ -6019,7 +6020,7 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="26" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B34" s="36">
         <f>Monthly_Cash!P23</f>
@@ -6046,7 +6047,7 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="26" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B35" s="36">
         <f>Monthly_Cash!Q23</f>
@@ -6073,7 +6074,7 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="26" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B36" s="36">
         <f>Monthly_Cash!R23</f>
@@ -6100,7 +6101,7 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="26" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B37" s="36">
         <f>Monthly_Cash!S23</f>
@@ -6127,7 +6128,7 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="26" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B38" s="36">
         <f>Monthly_Cash!T23</f>
@@ -6154,7 +6155,7 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="26" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="B39" s="36">
         <f>Monthly_Cash!U23</f>
@@ -6181,7 +6182,7 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="26" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B40" s="36">
         <f>Monthly_Cash!V23</f>
@@ -6208,7 +6209,7 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="26" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B41" s="36">
         <f>Monthly_Cash!W23</f>
@@ -6235,7 +6236,7 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="26" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B42" s="36">
         <f>Monthly_Cash!X23</f>
@@ -6262,7 +6263,7 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="26" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B43" s="36">
         <f>Monthly_Cash!Y23</f>
@@ -6289,7 +6290,7 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="26" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B44" s="36">
         <f>Monthly_Cash!Z23</f>
@@ -6316,7 +6317,7 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="26" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B45" s="36">
         <f>Monthly_Cash!AA23</f>
@@ -6343,7 +6344,7 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="26" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B46" s="36">
         <f>Monthly_Cash!AB23</f>
@@ -6370,7 +6371,7 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="26" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B47" s="36">
         <f>Monthly_Cash!AC23</f>
@@ -6397,7 +6398,7 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="26" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B48" s="36">
         <f>Monthly_Cash!AD23</f>
@@ -6424,7 +6425,7 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="26" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B49" s="36">
         <f>Monthly_Cash!AE23</f>
@@ -6451,7 +6452,7 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="26" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B50" s="36">
         <f>Monthly_Cash!AF23</f>
@@ -6478,7 +6479,7 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="26" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B51" s="36">
         <f>Monthly_Cash!AG23</f>
@@ -6505,7 +6506,7 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="26" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="B52" s="36">
         <f>Monthly_Cash!AH23</f>
@@ -6532,7 +6533,7 @@
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="26" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B53" s="36">
         <f>Monthly_Cash!AI23</f>
@@ -6559,7 +6560,7 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="26" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B54" s="36">
         <f>Monthly_Cash!AJ23</f>
@@ -6586,7 +6587,7 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="26" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B55" s="36">
         <f>Monthly_Cash!AK23</f>
@@ -6633,130 +6634,130 @@
   <sheetData>
     <row r="1" spans="1:3" ht="33">
       <c r="A1" s="81" t="s">
-        <v>20</v>
+        <v>407</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="82" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B2" s="82" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="83" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B3" s="83">
         <v>25000</v>
       </c>
       <c r="C3" s="83" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="84" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4" s="84">
         <v>500</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="83" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B5" s="83">
         <v>24500</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="84" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B6" s="84">
         <v>29500</v>
       </c>
       <c r="C6" s="84" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="83" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B7" s="83">
         <v>93500</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="84" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" s="84">
         <v>269000</v>
       </c>
       <c r="C8" s="84" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="83" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B9" s="83">
         <v>442000</v>
       </c>
       <c r="C9" s="83" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="84" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B10" s="84">
         <v>34950</v>
       </c>
       <c r="C10" s="84" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="83" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B11" s="83">
         <v>120320</v>
       </c>
       <c r="C11" s="83" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="84" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B12" s="84">
         <v>169300</v>
       </c>
       <c r="C12" s="84" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -6779,7 +6780,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="33">
       <c r="A1" s="81" t="s">
-        <v>40</v>
+        <v>408</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
@@ -6789,162 +6790,162 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="82" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="82" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="82" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="82" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="82" t="s">
+      <c r="F2" s="82" t="s">
         <v>42</v>
-      </c>
-      <c r="C2" s="82" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="82" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="82" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" s="82" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="28">
       <c r="A3" s="83" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="83" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="83" t="s">
+      <c r="F3" s="83" t="s">
         <v>48</v>
-      </c>
-      <c r="C3" s="83" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="83" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" s="83" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="83" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="84" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="84" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="84" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="84" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="84" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="F4" s="84" t="s">
         <v>54</v>
-      </c>
-      <c r="C4" s="84" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="84" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="84" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="84" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="83" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="83" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="83" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="83" t="s">
         <v>59</v>
-      </c>
-      <c r="B5" s="83" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="83" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="83" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" s="83" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" s="83" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="84" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="84" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="84" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="84" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="F6" s="84" t="s">
         <v>65</v>
-      </c>
-      <c r="C6" s="84" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="84" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" s="84" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="84" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="83" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="83" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="83" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="83" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="83" t="s">
+      <c r="F7" s="83" t="s">
         <v>71</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>72</v>
-      </c>
-      <c r="D7" s="83" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="83" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" s="83" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="84" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="84" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="84" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="84" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="84" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="84" t="s">
+      <c r="F8" s="84" t="s">
         <v>77</v>
-      </c>
-      <c r="C8" s="84" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="84" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" s="84" t="s">
-        <v>80</v>
-      </c>
-      <c r="F8" s="84" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="83" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="83" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="83" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="83" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="83" t="s">
+      <c r="F9" s="83" t="s">
         <v>83</v>
-      </c>
-      <c r="C9" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D9" s="83" t="s">
-        <v>85</v>
-      </c>
-      <c r="E9" s="83" t="s">
-        <v>86</v>
-      </c>
-      <c r="F9" s="83" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -6965,7 +6966,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="33">
       <c r="A1" s="81" t="s">
-        <v>88</v>
+        <v>409</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
@@ -6974,87 +6975,87 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="82" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B2" s="82" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D2" s="82" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="83" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B3" s="83" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C3" s="83" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D3" s="83" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E3" s="83" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="84" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B4" s="84" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D4" s="84" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="83" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D5" s="83" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E5" s="83" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="84" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B6" s="84" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C6" s="84" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D6" s="84" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E6" s="84" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -7075,7 +7076,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33">
       <c r="A1" s="81" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
@@ -7083,86 +7084,86 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="82" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" s="82" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D2" s="82" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="83" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B3" s="83" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C3" s="83" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D3" s="83" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="84" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B4" s="84" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D4" s="84" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="83" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D5" s="83" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="84" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B6" s="84" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C6" s="84" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D6" s="84" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="83" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D7" s="83" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -7183,7 +7184,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20">
       <c r="A1" s="87" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -7201,27 +7202,27 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="28">
       <c r="A4" s="5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B4" s="6">
         <v>25000</v>
@@ -7233,15 +7234,15 @@
         <v>0</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B5" s="6">
         <v>0</v>
@@ -7253,15 +7254,15 @@
         <v>0</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B6" s="7">
         <v>0.19</v>
@@ -7273,15 +7274,15 @@
         <v>0.19</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B7" s="7">
         <v>0.1</v>
@@ -7293,15 +7294,15 @@
         <v>0.15</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B8" s="6">
         <v>1600</v>
@@ -7313,15 +7314,15 @@
         <v>3200</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="42">
       <c r="A9" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B9" s="6">
         <v>2500</v>
@@ -7333,15 +7334,15 @@
         <v>5000</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="5" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B10" s="6">
         <v>0</v>
@@ -7353,15 +7354,15 @@
         <v>9000</v>
       </c>
       <c r="E10" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B11" s="6">
         <v>2000</v>
@@ -7373,15 +7374,15 @@
         <v>5000</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B12" s="6">
         <v>2000</v>
@@ -7393,15 +7394,15 @@
         <v>15000</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B13" s="6">
         <v>10000</v>
@@ -7413,15 +7414,15 @@
         <v>25000</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B14" s="7">
         <v>0.45</v>
@@ -7433,15 +7434,15 @@
         <v>0.45</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="5" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B15" s="7">
         <v>1.25</v>
@@ -7453,15 +7454,15 @@
         <v>1.25</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="5" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B16" s="8">
         <v>102</v>
@@ -7473,15 +7474,15 @@
         <v>140</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28">
       <c r="A17" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B17" s="6">
         <v>900</v>
@@ -7493,35 +7494,35 @@
         <v>900</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="42">
       <c r="A18" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B19" s="10">
         <v>0.3</v>
@@ -7533,27 +7534,27 @@
         <v>0.3</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="13" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
       <c r="E20" s="13"/>
       <c r="F20" s="20" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="15" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B21" s="16">
         <v>0.4</v>
@@ -7565,15 +7566,15 @@
         <v>0.2</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="15" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B22" s="16">
         <v>0.3</v>
@@ -7585,15 +7586,15 @@
         <v>0.3</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="15" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B23" s="16">
         <v>0.1</v>
@@ -7605,15 +7606,15 @@
         <v>0</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="15" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B24" s="16">
         <v>0.5</v>
@@ -7625,26 +7626,26 @@
         <v>0.2</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="15" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -7669,7 +7670,7 @@
   <sheetData>
     <row r="1" spans="1:40" ht="20">
       <c r="A1" s="87" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -7755,129 +7756,129 @@
     </row>
     <row r="3" spans="1:40" ht="28">
       <c r="A3" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="O3" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="U3" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="V3" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="X3" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="Y3" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="Z3" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="AA3" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="AB3" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="X3" s="4" t="s">
+      <c r="AC3" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="Y3" s="4" t="s">
+      <c r="AD3" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="Z3" s="4" t="s">
+      <c r="AE3" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="AA3" s="4" t="s">
+      <c r="AF3" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="AB3" s="4" t="s">
+      <c r="AG3" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="AC3" s="4" t="s">
+      <c r="AH3" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="AD3" s="4" t="s">
+      <c r="AI3" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="AE3" s="4" t="s">
+      <c r="AJ3" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="AF3" s="4" t="s">
+      <c r="AK3" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="AG3" s="4" t="s">
+      <c r="AL3" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="AH3" s="4" t="s">
+      <c r="AM3" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="AI3" s="4" t="s">
+      <c r="AN3" s="4" t="s">
         <v>228</v>
-      </c>
-      <c r="AJ3" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="AK3" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="AL3" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="AM3" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="AN3" s="4" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:40">
       <c r="A4" s="29" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B4" s="29">
         <v>1</v>
@@ -7886,7 +7887,7 @@
         <v>12500</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E4" s="31">
         <f>IF(Schedule_Inputs!$C$4="Blueprint",$C4*IF(1-Schedule_Inputs!$B$4=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$4=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$4=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$4="Launch",$C4*IF(1-Schedule_Inputs!$B$4=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$4=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$4=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$4=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$4="Office Setup",$C4*IF(1-Schedule_Inputs!$B$4=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$4=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$4=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$4="Monthly",Schedule_Inputs!$C$4="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$4,MOD(1-Schedule_Inputs!$B$4,Schedule_Inputs!$E$4)=0,(1-Schedule_Inputs!$B$4)/Schedule_Inputs!$E$4&lt;Schedule_Inputs!$D$4),$C4/Schedule_Inputs!$D$4,0),0))))</f>
@@ -8035,7 +8036,7 @@
     </row>
     <row r="5" spans="1:40">
       <c r="A5" s="29" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B5" s="29">
         <v>1</v>
@@ -8044,7 +8045,7 @@
         <v>12500</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E5" s="31">
         <f>IF(Schedule_Inputs!$C$5="Blueprint",$C5*IF(1-Schedule_Inputs!$B$5=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$5=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$5=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$5="Launch",$C5*IF(1-Schedule_Inputs!$B$5=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$5=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$5=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$5=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$5="Office Setup",$C5*IF(1-Schedule_Inputs!$B$5=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$5=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$5=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$5="Monthly",Schedule_Inputs!$C$5="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$5,MOD(1-Schedule_Inputs!$B$5,Schedule_Inputs!$E$5)=0,(1-Schedule_Inputs!$B$5)/Schedule_Inputs!$E$5&lt;Schedule_Inputs!$D$5),$C5/Schedule_Inputs!$D$5,0),0))))</f>
@@ -8193,7 +8194,7 @@
     </row>
     <row r="6" spans="1:40">
       <c r="A6" s="29" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B6" s="29">
         <v>1</v>
@@ -8202,7 +8203,7 @@
         <v>29500</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E6" s="31">
         <f>IF(Schedule_Inputs!$C$6="Blueprint",$C6*IF(1-Schedule_Inputs!$B$6=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$6=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$6=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$6="Launch",$C6*IF(1-Schedule_Inputs!$B$6=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$6=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$6=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$6=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$6="Office Setup",$C6*IF(1-Schedule_Inputs!$B$6=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$6=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$6=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$6="Monthly",Schedule_Inputs!$C$6="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$6,MOD(1-Schedule_Inputs!$B$6,Schedule_Inputs!$E$6)=0,(1-Schedule_Inputs!$B$6)/Schedule_Inputs!$E$6&lt;Schedule_Inputs!$D$6),$C6/Schedule_Inputs!$D$6,0),0))))</f>
@@ -8351,7 +8352,7 @@
     </row>
     <row r="7" spans="1:40">
       <c r="A7" s="29" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B7" s="29">
         <v>1</v>
@@ -8360,7 +8361,7 @@
         <v>15000</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E7" s="31">
         <f>IF(Schedule_Inputs!$C$7="Blueprint",$C7*IF(1-Schedule_Inputs!$B$7=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$7=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$7=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$7="Launch",$C7*IF(1-Schedule_Inputs!$B$7=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$7=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$7=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$7=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$7="Office Setup",$C7*IF(1-Schedule_Inputs!$B$7=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$7=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$7=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$7="Monthly",Schedule_Inputs!$C$7="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$7,MOD(1-Schedule_Inputs!$B$7,Schedule_Inputs!$E$7)=0,(1-Schedule_Inputs!$B$7)/Schedule_Inputs!$E$7&lt;Schedule_Inputs!$D$7),$C7/Schedule_Inputs!$D$7,0),0))))</f>
@@ -8509,7 +8510,7 @@
     </row>
     <row r="8" spans="1:40">
       <c r="A8" s="29" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B8" s="29">
         <v>1</v>
@@ -8518,7 +8519,7 @@
         <v>13500</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E8" s="31">
         <f>IF(Schedule_Inputs!$C$8="Blueprint",$C8*IF(1-Schedule_Inputs!$B$8=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$8=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$8=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$8="Launch",$C8*IF(1-Schedule_Inputs!$B$8=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$8=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$8=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$8=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$8="Office Setup",$C8*IF(1-Schedule_Inputs!$B$8=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$8=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$8=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$8="Monthly",Schedule_Inputs!$C$8="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$8,MOD(1-Schedule_Inputs!$B$8,Schedule_Inputs!$E$8)=0,(1-Schedule_Inputs!$B$8)/Schedule_Inputs!$E$8&lt;Schedule_Inputs!$D$8),$C8/Schedule_Inputs!$D$8,0),0))))</f>
@@ -8667,7 +8668,7 @@
     </row>
     <row r="9" spans="1:40">
       <c r="A9" s="29" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B9" s="29">
         <v>1</v>
@@ -8676,7 +8677,7 @@
         <v>10500</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E9" s="31">
         <f>IF(Schedule_Inputs!$C$9="Blueprint",$C9*IF(1-Schedule_Inputs!$B$9=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$9=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$9=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$9="Launch",$C9*IF(1-Schedule_Inputs!$B$9=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$9=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$9=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$9=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$9="Office Setup",$C9*IF(1-Schedule_Inputs!$B$9=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$9=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$9=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$9="Monthly",Schedule_Inputs!$C$9="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$9,MOD(1-Schedule_Inputs!$B$9,Schedule_Inputs!$E$9)=0,(1-Schedule_Inputs!$B$9)/Schedule_Inputs!$E$9&lt;Schedule_Inputs!$D$9),$C9/Schedule_Inputs!$D$9,0),0))))</f>
@@ -8825,7 +8826,7 @@
     </row>
     <row r="10" spans="1:40">
       <c r="A10" s="29" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B10" s="29">
         <v>2</v>
@@ -8834,7 +8835,7 @@
         <v>21000</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E10" s="31">
         <f>IF(Schedule_Inputs!$C$10="Blueprint",$C10*IF(1-Schedule_Inputs!$B$10=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$10=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$10=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$10="Launch",$C10*IF(1-Schedule_Inputs!$B$10=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$10=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$10=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$10=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$10="Office Setup",$C10*IF(1-Schedule_Inputs!$B$10=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$10=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$10=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$10="Monthly",Schedule_Inputs!$C$10="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$10,MOD(1-Schedule_Inputs!$B$10,Schedule_Inputs!$E$10)=0,(1-Schedule_Inputs!$B$10)/Schedule_Inputs!$E$10&lt;Schedule_Inputs!$D$10),$C10/Schedule_Inputs!$D$10,0),0))))</f>
@@ -8983,7 +8984,7 @@
     </row>
     <row r="11" spans="1:40">
       <c r="A11" s="29" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B11" s="29">
         <v>2</v>
@@ -8992,7 +8993,7 @@
         <v>21000</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E11" s="31">
         <f>IF(Schedule_Inputs!$C$11="Blueprint",$C11*IF(1-Schedule_Inputs!$B$11=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$11=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$11=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$11="Launch",$C11*IF(1-Schedule_Inputs!$B$11=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$11=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$11=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$11=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$11="Office Setup",$C11*IF(1-Schedule_Inputs!$B$11=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$11=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$11=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$11="Monthly",Schedule_Inputs!$C$11="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$11,MOD(1-Schedule_Inputs!$B$11,Schedule_Inputs!$E$11)=0,(1-Schedule_Inputs!$B$11)/Schedule_Inputs!$E$11&lt;Schedule_Inputs!$D$11),$C11/Schedule_Inputs!$D$11,0),0))))</f>
@@ -9141,7 +9142,7 @@
     </row>
     <row r="12" spans="1:40">
       <c r="A12" s="29" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B12" s="29">
         <v>2</v>
@@ -9150,7 +9151,7 @@
         <v>21000</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E12" s="31">
         <f>IF(Schedule_Inputs!$C$12="Blueprint",$C12*IF(1-Schedule_Inputs!$B$12=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$12=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$12=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$12="Launch",$C12*IF(1-Schedule_Inputs!$B$12=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$12=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$12=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$12=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$12="Office Setup",$C12*IF(1-Schedule_Inputs!$B$12=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$12=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$12=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$12="Monthly",Schedule_Inputs!$C$12="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$12,MOD(1-Schedule_Inputs!$B$12,Schedule_Inputs!$E$12)=0,(1-Schedule_Inputs!$B$12)/Schedule_Inputs!$E$12&lt;Schedule_Inputs!$D$12),$C12/Schedule_Inputs!$D$12,0),0))))</f>
@@ -9299,7 +9300,7 @@
     </row>
     <row r="13" spans="1:40">
       <c r="A13" s="29" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B13" s="29">
         <v>2</v>
@@ -9308,7 +9309,7 @@
         <v>50000</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E13" s="31">
         <f>IF(Schedule_Inputs!$C$13="Blueprint",$C13*IF(1-Schedule_Inputs!$B$13=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$13=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$13=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$13="Launch",$C13*IF(1-Schedule_Inputs!$B$13=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$13=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$13=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$13=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$13="Office Setup",$C13*IF(1-Schedule_Inputs!$B$13=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$13=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$13=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$13="Monthly",Schedule_Inputs!$C$13="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$13,MOD(1-Schedule_Inputs!$B$13,Schedule_Inputs!$E$13)=0,(1-Schedule_Inputs!$B$13)/Schedule_Inputs!$E$13&lt;Schedule_Inputs!$D$13),$C13/Schedule_Inputs!$D$13,0),0))))</f>
@@ -9457,7 +9458,7 @@
     </row>
     <row r="14" spans="1:40">
       <c r="A14" s="29" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B14" s="29">
         <v>2</v>
@@ -9466,7 +9467,7 @@
         <v>50000</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E14" s="31">
         <f>IF(Schedule_Inputs!$C$14="Blueprint",$C14*IF(1-Schedule_Inputs!$B$14=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$14=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$14=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$14="Launch",$C14*IF(1-Schedule_Inputs!$B$14=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$14=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$14=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$14=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$14="Office Setup",$C14*IF(1-Schedule_Inputs!$B$14=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$14=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$14=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$14="Monthly",Schedule_Inputs!$C$14="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$14,MOD(1-Schedule_Inputs!$B$14,Schedule_Inputs!$E$14)=0,(1-Schedule_Inputs!$B$14)/Schedule_Inputs!$E$14&lt;Schedule_Inputs!$D$14),$C14/Schedule_Inputs!$D$14,0),0))))</f>
@@ -9615,7 +9616,7 @@
     </row>
     <row r="15" spans="1:40">
       <c r="A15" s="29" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B15" s="29">
         <v>2</v>
@@ -9624,7 +9625,7 @@
         <v>25000</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E15" s="31">
         <f>IF(Schedule_Inputs!$C$15="Blueprint",$C15*IF(1-Schedule_Inputs!$B$15=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$15=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$15=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$15="Launch",$C15*IF(1-Schedule_Inputs!$B$15=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$15=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$15=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$15=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$15="Office Setup",$C15*IF(1-Schedule_Inputs!$B$15=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$15=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$15=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$15="Monthly",Schedule_Inputs!$C$15="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$15,MOD(1-Schedule_Inputs!$B$15,Schedule_Inputs!$E$15)=0,(1-Schedule_Inputs!$B$15)/Schedule_Inputs!$E$15&lt;Schedule_Inputs!$D$15),$C15/Schedule_Inputs!$D$15,0),0))))</f>
@@ -9773,7 +9774,7 @@
     </row>
     <row r="16" spans="1:40">
       <c r="A16" s="29" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B16" s="29">
         <v>2</v>
@@ -9782,7 +9783,7 @@
         <v>72000</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E16" s="31">
         <f>IF(Schedule_Inputs!$C$16="Blueprint",$C16*IF(1-Schedule_Inputs!$B$16=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$16=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$16=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$16="Launch",$C16*IF(1-Schedule_Inputs!$B$16=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$16=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$16=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$16=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$16="Office Setup",$C16*IF(1-Schedule_Inputs!$B$16=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$16=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$16=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$16="Monthly",Schedule_Inputs!$C$16="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$16,MOD(1-Schedule_Inputs!$B$16,Schedule_Inputs!$E$16)=0,(1-Schedule_Inputs!$B$16)/Schedule_Inputs!$E$16&lt;Schedule_Inputs!$D$16),$C16/Schedule_Inputs!$D$16,0),0))))</f>
@@ -9931,7 +9932,7 @@
     </row>
     <row r="17" spans="1:40">
       <c r="A17" s="29" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B17" s="29">
         <v>2</v>
@@ -9940,7 +9941,7 @@
         <v>9000</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E17" s="31">
         <f>IF(Schedule_Inputs!$C$17="Blueprint",$C17*IF(1-Schedule_Inputs!$B$17=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$17=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$17=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$17="Launch",$C17*IF(1-Schedule_Inputs!$B$17=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$17=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$17=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$17=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$17="Office Setup",$C17*IF(1-Schedule_Inputs!$B$17=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$17=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$17=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$17="Monthly",Schedule_Inputs!$C$17="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$17,MOD(1-Schedule_Inputs!$B$17,Schedule_Inputs!$E$17)=0,(1-Schedule_Inputs!$B$17)/Schedule_Inputs!$E$17&lt;Schedule_Inputs!$D$17),$C17/Schedule_Inputs!$D$17,0),0))))</f>
@@ -10089,7 +10090,7 @@
     </row>
     <row r="18" spans="1:40">
       <c r="A18" s="29" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B18" s="29">
         <v>3</v>
@@ -10098,7 +10099,7 @@
         <v>21000</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E18" s="31">
         <f>IF(Schedule_Inputs!$C$18="Blueprint",$C18*IF(1-Schedule_Inputs!$B$18=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$18=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$18=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$18="Launch",$C18*IF(1-Schedule_Inputs!$B$18=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$18=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$18=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$18=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$18="Office Setup",$C18*IF(1-Schedule_Inputs!$B$18=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$18=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$18=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$18="Monthly",Schedule_Inputs!$C$18="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$18,MOD(1-Schedule_Inputs!$B$18,Schedule_Inputs!$E$18)=0,(1-Schedule_Inputs!$B$18)/Schedule_Inputs!$E$18&lt;Schedule_Inputs!$D$18),$C18/Schedule_Inputs!$D$18,0),0))))</f>
@@ -10247,7 +10248,7 @@
     </row>
     <row r="19" spans="1:40">
       <c r="A19" s="29" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B19" s="29">
         <v>3</v>
@@ -10256,7 +10257,7 @@
         <v>21000</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E19" s="31">
         <f>IF(Schedule_Inputs!$C$19="Blueprint",$C19*IF(1-Schedule_Inputs!$B$19=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$19=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$19=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$19="Launch",$C19*IF(1-Schedule_Inputs!$B$19=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$19=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$19=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$19=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$19="Office Setup",$C19*IF(1-Schedule_Inputs!$B$19=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$19=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$19=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$19="Monthly",Schedule_Inputs!$C$19="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$19,MOD(1-Schedule_Inputs!$B$19,Schedule_Inputs!$E$19)=0,(1-Schedule_Inputs!$B$19)/Schedule_Inputs!$E$19&lt;Schedule_Inputs!$D$19),$C19/Schedule_Inputs!$D$19,0),0))))</f>
@@ -10405,7 +10406,7 @@
     </row>
     <row r="20" spans="1:40">
       <c r="A20" s="29" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B20" s="29">
         <v>3</v>
@@ -10414,7 +10415,7 @@
         <v>21000</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E20" s="31">
         <f>IF(Schedule_Inputs!$C$20="Blueprint",$C20*IF(1-Schedule_Inputs!$B$20=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$20=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$20=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$20="Launch",$C20*IF(1-Schedule_Inputs!$B$20=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$20=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$20=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$20=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$20="Office Setup",$C20*IF(1-Schedule_Inputs!$B$20=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$20=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$20=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$20="Monthly",Schedule_Inputs!$C$20="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$20,MOD(1-Schedule_Inputs!$B$20,Schedule_Inputs!$E$20)=0,(1-Schedule_Inputs!$B$20)/Schedule_Inputs!$E$20&lt;Schedule_Inputs!$D$20),$C20/Schedule_Inputs!$D$20,0),0))))</f>
@@ -10563,7 +10564,7 @@
     </row>
     <row r="21" spans="1:40">
       <c r="A21" s="29" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B21" s="29">
         <v>3</v>
@@ -10572,7 +10573,7 @@
         <v>21000</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E21" s="31">
         <f>IF(Schedule_Inputs!$C$21="Blueprint",$C21*IF(1-Schedule_Inputs!$B$21=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$21=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$21=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$21="Launch",$C21*IF(1-Schedule_Inputs!$B$21=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$21=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$21=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$21=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$21="Office Setup",$C21*IF(1-Schedule_Inputs!$B$21=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$21=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$21=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$21="Monthly",Schedule_Inputs!$C$21="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$21,MOD(1-Schedule_Inputs!$B$21,Schedule_Inputs!$E$21)=0,(1-Schedule_Inputs!$B$21)/Schedule_Inputs!$E$21&lt;Schedule_Inputs!$D$21),$C21/Schedule_Inputs!$D$21,0),0))))</f>
@@ -10721,7 +10722,7 @@
     </row>
     <row r="22" spans="1:40">
       <c r="A22" s="29" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B22" s="29">
         <v>3</v>
@@ -10730,7 +10731,7 @@
         <v>55000</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E22" s="31">
         <f>IF(Schedule_Inputs!$C$22="Blueprint",$C22*IF(1-Schedule_Inputs!$B$22=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$22=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$22=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$22="Launch",$C22*IF(1-Schedule_Inputs!$B$22=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$22=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$22=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$22=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$22="Office Setup",$C22*IF(1-Schedule_Inputs!$B$22=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$22=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$22=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$22="Monthly",Schedule_Inputs!$C$22="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$22,MOD(1-Schedule_Inputs!$B$22,Schedule_Inputs!$E$22)=0,(1-Schedule_Inputs!$B$22)/Schedule_Inputs!$E$22&lt;Schedule_Inputs!$D$22),$C22/Schedule_Inputs!$D$22,0),0))))</f>
@@ -10879,7 +10880,7 @@
     </row>
     <row r="23" spans="1:40">
       <c r="A23" s="29" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="B23" s="29">
         <v>3</v>
@@ -10888,7 +10889,7 @@
         <v>55000</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E23" s="31">
         <f>IF(Schedule_Inputs!$C$23="Blueprint",$C23*IF(1-Schedule_Inputs!$B$23=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$23=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$23=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$23="Launch",$C23*IF(1-Schedule_Inputs!$B$23=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$23=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$23=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$23=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$23="Office Setup",$C23*IF(1-Schedule_Inputs!$B$23=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$23=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$23=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$23="Monthly",Schedule_Inputs!$C$23="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$23,MOD(1-Schedule_Inputs!$B$23,Schedule_Inputs!$E$23)=0,(1-Schedule_Inputs!$B$23)/Schedule_Inputs!$E$23&lt;Schedule_Inputs!$D$23),$C23/Schedule_Inputs!$D$23,0),0))))</f>
@@ -11037,7 +11038,7 @@
     </row>
     <row r="24" spans="1:40">
       <c r="A24" s="29" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B24" s="29">
         <v>3</v>
@@ -11046,7 +11047,7 @@
         <v>28000</v>
       </c>
       <c r="D24" s="31" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E24" s="31">
         <f>IF(Schedule_Inputs!$C$24="Blueprint",$C24*IF(1-Schedule_Inputs!$B$24=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$24=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$24=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$24="Launch",$C24*IF(1-Schedule_Inputs!$B$24=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$24=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$24=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$24=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$24="Office Setup",$C24*IF(1-Schedule_Inputs!$B$24=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$24=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$24=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$24="Monthly",Schedule_Inputs!$C$24="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$24,MOD(1-Schedule_Inputs!$B$24,Schedule_Inputs!$E$24)=0,(1-Schedule_Inputs!$B$24)/Schedule_Inputs!$E$24&lt;Schedule_Inputs!$D$24),$C24/Schedule_Inputs!$D$24,0),0))))</f>
@@ -11195,7 +11196,7 @@
     </row>
     <row r="25" spans="1:40">
       <c r="A25" s="29" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B25" s="29">
         <v>3</v>
@@ -11204,7 +11205,7 @@
         <v>28000</v>
       </c>
       <c r="D25" s="31" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E25" s="31">
         <f>IF(Schedule_Inputs!$C$25="Blueprint",$C25*IF(1-Schedule_Inputs!$B$25=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$25=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$25=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$25="Launch",$C25*IF(1-Schedule_Inputs!$B$25=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$25=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$25=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$25=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$25="Office Setup",$C25*IF(1-Schedule_Inputs!$B$25=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$25=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$25=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$25="Monthly",Schedule_Inputs!$C$25="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$25,MOD(1-Schedule_Inputs!$B$25,Schedule_Inputs!$E$25)=0,(1-Schedule_Inputs!$B$25)/Schedule_Inputs!$E$25&lt;Schedule_Inputs!$D$25),$C25/Schedule_Inputs!$D$25,0),0))))</f>
@@ -11353,7 +11354,7 @@
     </row>
     <row r="26" spans="1:40">
       <c r="A26" s="29" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B26" s="29">
         <v>3</v>
@@ -11362,7 +11363,7 @@
         <v>144000</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E26" s="31">
         <f>IF(Schedule_Inputs!$C$26="Blueprint",$C26*IF(1-Schedule_Inputs!$B$26=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$26=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$26=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$26="Launch",$C26*IF(1-Schedule_Inputs!$B$26=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$26=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$26=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$26=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$26="Office Setup",$C26*IF(1-Schedule_Inputs!$B$26=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$26=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$26=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$26="Monthly",Schedule_Inputs!$C$26="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$26,MOD(1-Schedule_Inputs!$B$26,Schedule_Inputs!$E$26)=0,(1-Schedule_Inputs!$B$26)/Schedule_Inputs!$E$26&lt;Schedule_Inputs!$D$26),$C26/Schedule_Inputs!$D$26,0),0))))</f>
@@ -11511,7 +11512,7 @@
     </row>
     <row r="27" spans="1:40">
       <c r="A27" s="29" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B27" s="29">
         <v>3</v>
@@ -11520,7 +11521,7 @@
         <v>48000</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E27" s="31">
         <f>IF(Schedule_Inputs!$C$27="Blueprint",$C27*IF(1-Schedule_Inputs!$B$27=0,Assumptions!$B$21,IF(1-Schedule_Inputs!$B$27=1,Assumptions!$C$21,IF(1-Schedule_Inputs!$B$27=2,Assumptions!$D$21,0))),IF(Schedule_Inputs!$C$27="Launch",$C27*IF(1-Schedule_Inputs!$B$27=0,Assumptions!$B$22,IF(1-Schedule_Inputs!$B$27=1,Assumptions!$C$22,IF(1-Schedule_Inputs!$B$27=2,Assumptions!$D$22,IF(1-Schedule_Inputs!$B$27=3,Assumptions!$B$23,0)))),IF(Schedule_Inputs!$C$27="Office Setup",$C27*IF(1-Schedule_Inputs!$B$27=0,Assumptions!$B$24,IF(1-Schedule_Inputs!$B$27=1,Assumptions!$C$24,IF(1-Schedule_Inputs!$B$27=2,Assumptions!$D$24,0))),IF(OR(Schedule_Inputs!$C$27="Monthly",Schedule_Inputs!$C$27="Periodic"),IF(AND(1&gt;=Schedule_Inputs!$B$27,MOD(1-Schedule_Inputs!$B$27,Schedule_Inputs!$E$27)=0,(1-Schedule_Inputs!$B$27)/Schedule_Inputs!$E$27&lt;Schedule_Inputs!$D$27),$C27/Schedule_Inputs!$D$27,0),0))))</f>
@@ -11669,7 +11670,7 @@
     </row>
     <row r="28" spans="1:40">
       <c r="A28" s="32" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B28" s="32"/>
       <c r="C28" s="33">
@@ -11841,7 +11842,7 @@
   <sheetData>
     <row r="1" spans="1:37" ht="28" customHeight="1">
       <c r="A1" s="88" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -11921,120 +11922,120 @@
     </row>
     <row r="3" spans="1:37">
       <c r="A3" s="22" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B3" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="G3" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="H3" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="I3" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="J3" s="22" t="s">
         <v>201</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="K3" s="22" t="s">
         <v>202</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="L3" s="22" t="s">
         <v>203</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="M3" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="N3" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="J3" s="22" t="s">
+      <c r="O3" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="P3" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="L3" s="22" t="s">
+      <c r="Q3" s="22" t="s">
         <v>208</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="R3" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="N3" s="22" t="s">
+      <c r="S3" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="O3" s="22" t="s">
+      <c r="T3" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="P3" s="22" t="s">
+      <c r="U3" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="Q3" s="22" t="s">
+      <c r="V3" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="R3" s="22" t="s">
+      <c r="W3" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="S3" s="22" t="s">
+      <c r="X3" s="22" t="s">
         <v>215</v>
       </c>
-      <c r="T3" s="22" t="s">
+      <c r="Y3" s="22" t="s">
         <v>216</v>
       </c>
-      <c r="U3" s="22" t="s">
+      <c r="Z3" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="V3" s="22" t="s">
+      <c r="AA3" s="22" t="s">
         <v>218</v>
       </c>
-      <c r="W3" s="22" t="s">
+      <c r="AB3" s="22" t="s">
         <v>219</v>
       </c>
-      <c r="X3" s="22" t="s">
+      <c r="AC3" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="Y3" s="22" t="s">
+      <c r="AD3" s="22" t="s">
         <v>221</v>
       </c>
-      <c r="Z3" s="22" t="s">
+      <c r="AE3" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="AA3" s="22" t="s">
+      <c r="AF3" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="AB3" s="22" t="s">
+      <c r="AG3" s="22" t="s">
         <v>224</v>
       </c>
-      <c r="AC3" s="22" t="s">
+      <c r="AH3" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="AD3" s="22" t="s">
+      <c r="AI3" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="AE3" s="22" t="s">
+      <c r="AJ3" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="AF3" s="22" t="s">
+      <c r="AK3" s="22" t="s">
         <v>228</v>
-      </c>
-      <c r="AG3" s="22" t="s">
-        <v>229</v>
-      </c>
-      <c r="AH3" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="AI3" s="22" t="s">
-        <v>231</v>
-      </c>
-      <c r="AJ3" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="AK3" s="22" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:37">
       <c r="A4" s="35" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B4" s="36">
         <f>Contract_Cash!E28</f>
@@ -12183,7 +12184,7 @@
     </row>
     <row r="5" spans="1:37">
       <c r="A5" s="35" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B5" s="36">
         <f>B4*Assumptions!B6</f>
@@ -12332,7 +12333,7 @@
     </row>
     <row r="6" spans="1:37">
       <c r="A6" s="35" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B6" s="36">
         <f>0</f>
@@ -12481,7 +12482,7 @@
     </row>
     <row r="7" spans="1:37">
       <c r="A7" s="35" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B7" s="36">
         <f t="shared" ref="B7:AK7" si="1">B4+B5-B6</f>
@@ -12630,7 +12631,7 @@
     </row>
     <row r="8" spans="1:37">
       <c r="A8" s="35" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B8" s="36">
         <f>B4*Assumptions!B7</f>
@@ -12779,7 +12780,7 @@
     </row>
     <row r="9" spans="1:37">
       <c r="A9" s="35" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B9" s="36">
         <f>Assumptions!B8</f>
@@ -12928,7 +12929,7 @@
     </row>
     <row r="10" spans="1:37">
       <c r="A10" s="35" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B10" s="36">
         <f>Assumptions!B9</f>
@@ -13077,7 +13078,7 @@
     </row>
     <row r="11" spans="1:37">
       <c r="A11" s="35" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B11" s="36">
         <f>Assumptions!B10</f>
@@ -13226,120 +13227,156 @@
     </row>
     <row r="12" spans="1:37">
       <c r="A12" s="35" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B12" s="36">
+        <f>Assumptions!$B$12*75%</f>
         <v>1500</v>
       </c>
       <c r="C12" s="36">
+        <f>Assumptions!$B$12*25%</f>
         <v>500</v>
       </c>
       <c r="D12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="E12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="F12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="G12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="H12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="I12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="J12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="K12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="L12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="M12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="N12" s="36">
+        <f>Assumptions!$C$12*50%</f>
         <v>4000</v>
       </c>
       <c r="O12" s="36">
+        <f>Assumptions!$C$12*25%</f>
         <v>2000</v>
       </c>
       <c r="P12" s="36">
+        <f>Assumptions!$C$12*25%</f>
         <v>2000</v>
       </c>
       <c r="Q12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="R12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="S12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="T12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="U12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="V12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="W12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="X12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="Y12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="Z12" s="36">
+        <f>Assumptions!$D$12/3</f>
         <v>5000</v>
       </c>
       <c r="AA12" s="36">
+        <f>Assumptions!$D$12/3</f>
         <v>5000</v>
       </c>
       <c r="AB12" s="36">
+        <f>Assumptions!$D$12/3</f>
         <v>5000</v>
       </c>
       <c r="AC12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AD12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AE12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AF12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AG12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AH12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AI12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AJ12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="AK12" s="36">
+        <f>0</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:37">
       <c r="A13" s="35" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B13" s="36">
         <f t="shared" ref="B13:AK13" si="2">B7-B8-B9-B10-B11-B12</f>
@@ -13488,7 +13525,7 @@
     </row>
     <row r="14" spans="1:37">
       <c r="A14" s="35" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B14" s="36">
         <f>Assumptions!B4</f>
@@ -13637,7 +13674,7 @@
     </row>
     <row r="15" spans="1:37">
       <c r="A15" s="35" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B15" s="36">
         <f>Assumptions!B5</f>
@@ -13786,7 +13823,7 @@
     </row>
     <row r="16" spans="1:37">
       <c r="A16" s="35" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B16" s="36">
         <f>0</f>
@@ -13935,7 +13972,7 @@
     </row>
     <row r="17" spans="1:37">
       <c r="A17" s="13" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B17" s="37">
         <f t="shared" ref="B17:AK17" si="4">B16+B13+B14</f>
@@ -14084,7 +14121,7 @@
     </row>
     <row r="18" spans="1:37">
       <c r="A18" s="35" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B18" s="36">
         <f>0</f>
@@ -14233,7 +14270,7 @@
     </row>
     <row r="19" spans="1:37">
       <c r="A19" s="38" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B19" s="39">
         <f t="shared" ref="B19:AK19" si="6">B18+B13+B15</f>
@@ -14382,7 +14419,7 @@
     </row>
     <row r="20" spans="1:37">
       <c r="A20" s="40" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B20" s="41">
         <f t="shared" ref="B20:AK20" si="7">B5</f>
@@ -14531,7 +14568,7 @@
     </row>
     <row r="21" spans="1:37">
       <c r="A21" s="40" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B21" s="41">
         <f>'Annual_P&amp;L'!B12/12</f>
@@ -14680,7 +14717,7 @@
     </row>
     <row r="22" spans="1:37">
       <c r="A22" s="40" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B22" s="41">
         <f>B21</f>
@@ -14829,7 +14866,7 @@
     </row>
     <row r="23" spans="1:37">
       <c r="A23" s="42" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B23" s="43">
         <f t="shared" ref="B23:AK23" si="9">B17-B20-B22</f>
@@ -14978,7 +15015,7 @@
     </row>
     <row r="24" spans="1:37">
       <c r="A24" s="42" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B24" s="43">
         <f t="shared" ref="B24:AK24" si="10">B19-B20-B22</f>
@@ -15127,7 +15164,7 @@
     </row>
     <row r="25" spans="1:37">
       <c r="A25" s="40" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B25" s="41">
         <f>Assumptions!B13</f>
@@ -15276,7 +15313,7 @@
     </row>
     <row r="26" spans="1:37">
       <c r="A26" s="38" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B26" s="39">
         <f t="shared" ref="B26:AK26" si="11">B23-B25</f>
@@ -15425,7 +15462,7 @@
     </row>
     <row r="27" spans="1:37">
       <c r="A27" s="38" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B27" s="39">
         <f t="shared" ref="B27:AK27" si="12">B24-B25</f>
@@ -15574,7 +15611,7 @@
     </row>
     <row r="28" spans="1:37">
       <c r="A28" s="40" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B28" s="44" t="str">
         <f t="shared" ref="B28:AK28" si="13">IF(B26&gt;=0,"OK","BELOW MIN")</f>
@@ -15723,7 +15760,7 @@
     </row>
     <row r="29" spans="1:37">
       <c r="A29" s="40" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B29" s="44" t="str">
         <f t="shared" ref="B29:AK29" si="14">IF(B27&gt;=0,"OK","BELOW MIN")</f>
@@ -15872,10 +15909,10 @@
     </row>
     <row r="30" spans="1:37" ht="14.5">
       <c r="A30" s="34" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B30" s="89" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C30" s="86"/>
       <c r="D30" s="86"/>
@@ -15941,7 +15978,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20">
       <c r="A1" s="87" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -15955,21 +15992,21 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="29" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B4" s="31">
         <f>SUMIF(Contract_Cash!$B$4:$B$27,1,Contract_Cash!$C$4:$C$27)</f>
@@ -15986,7 +16023,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="29" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B5" s="31">
         <f>B4*Assumptions!B7</f>
@@ -16003,7 +16040,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="29" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B6" s="31">
         <f>Assumptions!B8*12</f>
@@ -16020,7 +16057,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="29" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B7" s="31">
         <f>Assumptions!B9*12</f>
@@ -16037,7 +16074,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="29" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B8" s="31">
         <f>Assumptions!B10*12</f>
@@ -16054,7 +16091,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="29" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B9" s="31">
         <f>B4-B5-B6-B7-B8</f>
@@ -16071,7 +16108,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="29" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B10" s="31">
         <f>Assumptions!B11</f>
@@ -16088,7 +16125,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="29" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B11" s="31">
         <f>B9-B10</f>
@@ -16105,7 +16142,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="29" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B12" s="31">
         <f>MAX(0,B11*Assumptions!B19)</f>
@@ -16122,7 +16159,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="29" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B13" s="31">
         <f>B11-B12</f>
@@ -16139,10 +16176,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="29" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B14" s="90" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="C14" s="91"/>
       <c r="D14" s="92"/>

</xml_diff>